<commit_message>
Textile : sous-onglet Planning PE des mousses (avancement, calendrier par avion, forecast 12/24/36 mois par PN et par fournisseur, exports) à partir du fichier mensuel PE_MOUSSE
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QT8GhHjeho8wXovFt7nryP
</commit_message>
<xml_diff>
--- a/tests/fixtures/commandes_sap.xlsx
+++ b/tests/fixtures/commandes_sap.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1067,48 +1067,101 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>FM-1004</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CMD-0040</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>AC20</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>245</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>F031</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Fournisseur Tango</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="n">
+        <v>46357</v>
+      </c>
+      <c r="H15" s="1" t="n">
+        <v>46402</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>En cours</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>150</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" t="n">
+        <v>60</v>
+      </c>
+      <c r="M15" s="1" t="n">
+        <v>46297</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>FX-1003</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>CMD-0031</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>AC03</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D16" t="n">
         <v>246</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>F003</t>
         </is>
       </c>
-      <c r="G15" s="1" t="n">
+      <c r="G16" s="1" t="n">
         <v>46174</v>
       </c>
-      <c r="H15" s="1" t="n">
+      <c r="H16" s="1" t="n">
         <v>54424</v>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>En cours</t>
         </is>
       </c>
-      <c r="J15" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" t="n">
-        <v>1</v>
-      </c>
-      <c r="L15" t="n">
+      <c r="J16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" t="n">
         <v>13</v>
       </c>
-      <c r="M15" s="1" t="n">
+      <c r="M16" s="1" t="n">
         <v>46114</v>
       </c>
     </row>

</xml_diff>